<commit_message>
Added step to catch case where no entry has been provided for the highest level taxonomic rank
</commit_message>
<xml_diff>
--- a/test/fixtures/Test_format_bad_Seq.xlsx
+++ b/test/fixtures/Test_format_bad_Seq.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Documents/MyRepos/safedata_validator/test/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{379131E4-457F-3B45-A8ED-F2346D43F11C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3830178D-D4FD-2348-9DCE-6F7C8818B76C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1060" windowWidth="27860" windowHeight="15840" activeTab="3" xr2:uid="{819B57D8-7F20-471A-9405-EB60A28E68AA}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8163" uniqueCount="1439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8165" uniqueCount="1442">
   <si>
     <t>Kingdom</t>
   </si>
@@ -4349,6 +4349,15 @@
   </si>
   <si>
     <t>carneum</t>
+  </si>
+  <si>
+    <t>test that blank works instead of NA</t>
+  </si>
+  <si>
+    <t>Just Eukaryote fine</t>
+  </si>
+  <si>
+    <t>Kingdom without superkingdom doesn't work</t>
   </si>
 </sst>
 </file>
@@ -6564,8 +6573,8 @@
       <c r="H7" t="s">
         <v>1414</v>
       </c>
-      <c r="I7" t="s">
-        <v>7</v>
+      <c r="J7" t="s">
+        <v>1439</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -6664,7 +6673,7 @@
         <v>1435</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>1379</v>
       </c>
@@ -6672,7 +6681,7 @@
         <v>1370</v>
       </c>
       <c r="C11" t="s">
-        <v>1384</v>
+        <v>7</v>
       </c>
       <c r="D11" t="s">
         <v>1386</v>
@@ -6692,14 +6701,16 @@
       <c r="I11" t="s">
         <v>1430</v>
       </c>
-      <c r="J11" s="1"/>
+      <c r="J11" s="1" t="s">
+        <v>1440</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>1380</v>
       </c>
       <c r="B12" t="s">
-        <v>1370</v>
+        <v>7</v>
       </c>
       <c r="C12" t="s">
         <v>1384</v>
@@ -6721,6 +6732,9 @@
       </c>
       <c r="I12" t="s">
         <v>1436</v>
+      </c>
+      <c r="J12" t="s">
+        <v>1441</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">

</xml_diff>